<commit_message>
feat: prepare for Azure deployment
- Add Azure Static Web Apps config (staticwebapp.config.json)
- Add Emir Özçakıcı to logger dropdown, remove KaleMaden
- Sanitize logger field: strip project names (e.g. CEYHAN) from display
- Fix Excel template borders (SO4, Düşünceler columns)
- Fix Ruhsat adı format: CEYHAN - CYHN-33 KUYUSU
- Update sample tag auto-increment logic
</commit_message>
<xml_diff>
--- a/public/Numune_Teslim_Formu.xlsx
+++ b/public/Numune_Teslim_Formu.xlsx
@@ -105,7 +105,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="20">
+  <borders count="24">
     <border>
       <left/>
       <right/>
@@ -372,11 +372,46 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium"/>
+    </border>
+    <border>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
@@ -526,6 +561,18 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -979,7 +1026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:AE47"/>
+  <dimension ref="B3:AE47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.2"/>
   <cols>
     <col width="6.88671875" customWidth="1" min="1" max="1"/>
@@ -1006,8 +1053,6 @@
     <col width="33" customWidth="1" min="33" max="33"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
     <row r="3" ht="15.6" customHeight="1">
       <c r="AC3" s="50" t="n"/>
     </row>
@@ -1172,7 +1217,7 @@
           <t>XRF</t>
         </is>
       </c>
-      <c r="Y9" s="8" t="inlineStr">
+      <c r="Y9" s="54" t="inlineStr">
         <is>
           <t>SO4</t>
         </is>
@@ -1199,7 +1244,7 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="AD9" s="8" t="inlineStr">
+      <c r="AD9" s="15" t="inlineStr">
         <is>
           <t>DÜŞÜNCELER</t>
         </is>
@@ -1237,12 +1282,12 @@
       <c r="V10" s="17" t="n"/>
       <c r="W10" s="17" t="n"/>
       <c r="X10" s="26" t="n"/>
-      <c r="Y10" s="26" t="n"/>
+      <c r="Y10" s="55" t="n"/>
       <c r="Z10" s="17" t="n"/>
       <c r="AA10" s="17" t="n"/>
       <c r="AB10" s="17" t="n"/>
       <c r="AC10" s="17" t="n"/>
-      <c r="AD10" s="18" t="n"/>
+      <c r="AD10" s="55" t="n"/>
     </row>
     <row r="11" ht="24.9" customHeight="1">
       <c r="B11" s="46" t="inlineStr">
@@ -1276,12 +1321,12 @@
       <c r="V11" s="10" t="n"/>
       <c r="W11" s="10" t="n"/>
       <c r="X11" s="26" t="n"/>
-      <c r="Y11" s="26" t="n"/>
+      <c r="Y11" s="55" t="n"/>
       <c r="Z11" s="10" t="n"/>
       <c r="AA11" s="10" t="n"/>
       <c r="AB11" s="25" t="n"/>
       <c r="AC11" s="10" t="n"/>
-      <c r="AD11" s="19" t="n"/>
+      <c r="AD11" s="55" t="n"/>
     </row>
     <row r="12" ht="24.9" customHeight="1">
       <c r="B12" s="46" t="inlineStr">
@@ -1315,12 +1360,12 @@
       <c r="V12" s="10" t="n"/>
       <c r="W12" s="10" t="n"/>
       <c r="X12" s="26" t="n"/>
-      <c r="Y12" s="26" t="n"/>
+      <c r="Y12" s="55" t="n"/>
       <c r="Z12" s="10" t="n"/>
       <c r="AA12" s="10" t="n"/>
       <c r="AB12" s="25" t="n"/>
       <c r="AC12" s="10" t="n"/>
-      <c r="AD12" s="19" t="n"/>
+      <c r="AD12" s="55" t="n"/>
     </row>
     <row r="13" ht="24.9" customHeight="1">
       <c r="B13" s="46" t="inlineStr">
@@ -1354,12 +1399,12 @@
       <c r="V13" s="10" t="n"/>
       <c r="W13" s="10" t="n"/>
       <c r="X13" s="26" t="n"/>
-      <c r="Y13" s="26" t="n"/>
+      <c r="Y13" s="55" t="n"/>
       <c r="Z13" s="10" t="n"/>
       <c r="AA13" s="16" t="n"/>
       <c r="AB13" s="25" t="n"/>
       <c r="AC13" s="10" t="n"/>
-      <c r="AD13" s="19" t="n"/>
+      <c r="AD13" s="55" t="n"/>
     </row>
     <row r="14" ht="24.9" customHeight="1">
       <c r="B14" s="46" t="n"/>
@@ -1385,12 +1430,12 @@
       <c r="V14" s="10" t="n"/>
       <c r="W14" s="10" t="n"/>
       <c r="X14" s="26" t="n"/>
-      <c r="Y14" s="26" t="n"/>
+      <c r="Y14" s="55" t="n"/>
       <c r="Z14" s="10" t="n"/>
       <c r="AA14" s="10" t="n"/>
       <c r="AB14" s="25" t="n"/>
       <c r="AC14" s="10" t="n"/>
-      <c r="AD14" s="19" t="n"/>
+      <c r="AD14" s="55" t="n"/>
     </row>
     <row r="15" ht="24.9" customHeight="1">
       <c r="B15" s="46" t="n"/>
@@ -1416,12 +1461,12 @@
       <c r="V15" s="10" t="n"/>
       <c r="W15" s="10" t="n"/>
       <c r="X15" s="26" t="n"/>
-      <c r="Y15" s="26" t="n"/>
+      <c r="Y15" s="55" t="n"/>
       <c r="Z15" s="10" t="n"/>
       <c r="AA15" s="10" t="n"/>
       <c r="AB15" s="25" t="n"/>
       <c r="AC15" s="10" t="n"/>
-      <c r="AD15" s="19" t="n"/>
+      <c r="AD15" s="55" t="n"/>
     </row>
     <row r="16" ht="24.9" customHeight="1">
       <c r="B16" s="46" t="n"/>
@@ -1447,12 +1492,12 @@
       <c r="V16" s="10" t="n"/>
       <c r="W16" s="10" t="n"/>
       <c r="X16" s="26" t="n"/>
-      <c r="Y16" s="26" t="n"/>
+      <c r="Y16" s="55" t="n"/>
       <c r="Z16" s="10" t="n"/>
       <c r="AA16" s="16" t="n"/>
       <c r="AB16" s="25" t="n"/>
       <c r="AC16" s="10" t="n"/>
-      <c r="AD16" s="19" t="n"/>
+      <c r="AD16" s="55" t="n"/>
     </row>
     <row r="17" ht="24.9" customHeight="1">
       <c r="B17" s="46" t="n"/>
@@ -1478,12 +1523,12 @@
       <c r="V17" s="10" t="n"/>
       <c r="W17" s="10" t="n"/>
       <c r="X17" s="26" t="n"/>
-      <c r="Y17" s="26" t="n"/>
+      <c r="Y17" s="55" t="n"/>
       <c r="Z17" s="10" t="n"/>
       <c r="AA17" s="16" t="n"/>
       <c r="AB17" s="25" t="n"/>
       <c r="AC17" s="10" t="n"/>
-      <c r="AD17" s="19" t="n"/>
+      <c r="AD17" s="55" t="n"/>
     </row>
     <row r="18" ht="24.9" customHeight="1">
       <c r="B18" s="46" t="n"/>
@@ -1509,12 +1554,12 @@
       <c r="V18" s="10" t="n"/>
       <c r="W18" s="10" t="n"/>
       <c r="X18" s="26" t="n"/>
-      <c r="Y18" s="26" t="n"/>
+      <c r="Y18" s="55" t="n"/>
       <c r="Z18" s="10" t="n"/>
       <c r="AA18" s="10" t="n"/>
       <c r="AB18" s="25" t="n"/>
       <c r="AC18" s="10" t="n"/>
-      <c r="AD18" s="19" t="n"/>
+      <c r="AD18" s="55" t="n"/>
     </row>
     <row r="19" ht="24.9" customHeight="1">
       <c r="B19" s="46" t="n"/>
@@ -1540,12 +1585,12 @@
       <c r="V19" s="10" t="n"/>
       <c r="W19" s="10" t="n"/>
       <c r="X19" s="26" t="n"/>
-      <c r="Y19" s="26" t="n"/>
+      <c r="Y19" s="55" t="n"/>
       <c r="Z19" s="10" t="n"/>
       <c r="AA19" s="10" t="n"/>
       <c r="AB19" s="25" t="n"/>
       <c r="AC19" s="10" t="n"/>
-      <c r="AD19" s="19" t="n"/>
+      <c r="AD19" s="55" t="n"/>
     </row>
     <row r="20" ht="24.9" customHeight="1">
       <c r="B20" s="46" t="n"/>
@@ -1571,12 +1616,12 @@
       <c r="V20" s="10" t="n"/>
       <c r="W20" s="10" t="n"/>
       <c r="X20" s="26" t="n"/>
-      <c r="Y20" s="26" t="n"/>
+      <c r="Y20" s="55" t="n"/>
       <c r="Z20" s="10" t="n"/>
       <c r="AA20" s="10" t="n"/>
       <c r="AB20" s="25" t="n"/>
       <c r="AC20" s="10" t="n"/>
-      <c r="AD20" s="19" t="n"/>
+      <c r="AD20" s="55" t="n"/>
     </row>
     <row r="21" ht="24.9" customHeight="1">
       <c r="B21" s="46" t="n"/>
@@ -1602,12 +1647,12 @@
       <c r="V21" s="10" t="n"/>
       <c r="W21" s="10" t="n"/>
       <c r="X21" s="26" t="n"/>
-      <c r="Y21" s="26" t="n"/>
+      <c r="Y21" s="55" t="n"/>
       <c r="Z21" s="10" t="n"/>
       <c r="AA21" s="10" t="n"/>
       <c r="AB21" s="25" t="n"/>
       <c r="AC21" s="10" t="n"/>
-      <c r="AD21" s="19" t="n"/>
+      <c r="AD21" s="55" t="n"/>
     </row>
     <row r="22" ht="24.9" customHeight="1">
       <c r="B22" s="46" t="n"/>
@@ -1633,12 +1678,12 @@
       <c r="V22" s="10" t="n"/>
       <c r="W22" s="10" t="n"/>
       <c r="X22" s="26" t="n"/>
-      <c r="Y22" s="26" t="n"/>
+      <c r="Y22" s="55" t="n"/>
       <c r="Z22" s="10" t="n"/>
       <c r="AA22" s="10" t="n"/>
       <c r="AB22" s="25" t="n"/>
       <c r="AC22" s="10" t="n"/>
-      <c r="AD22" s="19" t="n"/>
+      <c r="AD22" s="55" t="n"/>
     </row>
     <row r="23" ht="24.9" customHeight="1">
       <c r="B23" s="46" t="n"/>
@@ -1664,12 +1709,12 @@
       <c r="V23" s="10" t="n"/>
       <c r="W23" s="10" t="n"/>
       <c r="X23" s="26" t="n"/>
-      <c r="Y23" s="26" t="n"/>
+      <c r="Y23" s="55" t="n"/>
       <c r="Z23" s="10" t="n"/>
       <c r="AA23" s="10" t="n"/>
       <c r="AB23" s="25" t="n"/>
       <c r="AC23" s="10" t="n"/>
-      <c r="AD23" s="19" t="n"/>
+      <c r="AD23" s="55" t="n"/>
     </row>
     <row r="24" ht="24.9" customHeight="1">
       <c r="B24" s="46" t="n"/>
@@ -1695,12 +1740,12 @@
       <c r="V24" s="10" t="n"/>
       <c r="W24" s="10" t="n"/>
       <c r="X24" s="26" t="n"/>
-      <c r="Y24" s="26" t="n"/>
+      <c r="Y24" s="55" t="n"/>
       <c r="Z24" s="10" t="n"/>
       <c r="AA24" s="10" t="n"/>
       <c r="AB24" s="25" t="n"/>
       <c r="AC24" s="10" t="n"/>
-      <c r="AD24" s="19" t="n"/>
+      <c r="AD24" s="55" t="n"/>
     </row>
     <row r="25" ht="24.9" customHeight="1">
       <c r="B25" s="46" t="n"/>
@@ -1726,12 +1771,12 @@
       <c r="V25" s="10" t="n"/>
       <c r="W25" s="10" t="n"/>
       <c r="X25" s="26" t="n"/>
-      <c r="Y25" s="26" t="n"/>
+      <c r="Y25" s="55" t="n"/>
       <c r="Z25" s="10" t="n"/>
       <c r="AA25" s="10" t="n"/>
       <c r="AB25" s="25" t="n"/>
       <c r="AC25" s="10" t="n"/>
-      <c r="AD25" s="19" t="n"/>
+      <c r="AD25" s="55" t="n"/>
     </row>
     <row r="26" ht="24.9" customHeight="1">
       <c r="B26" s="46" t="n"/>
@@ -1757,12 +1802,12 @@
       <c r="V26" s="10" t="n"/>
       <c r="W26" s="10" t="n"/>
       <c r="X26" s="26" t="n"/>
-      <c r="Y26" s="26" t="n"/>
+      <c r="Y26" s="55" t="n"/>
       <c r="Z26" s="10" t="n"/>
       <c r="AA26" s="10" t="n"/>
       <c r="AB26" s="25" t="n"/>
       <c r="AC26" s="10" t="n"/>
-      <c r="AD26" s="19" t="n"/>
+      <c r="AD26" s="55" t="n"/>
     </row>
     <row r="27" ht="24.9" customHeight="1">
       <c r="B27" s="46" t="n"/>
@@ -1788,12 +1833,12 @@
       <c r="V27" s="10" t="n"/>
       <c r="W27" s="10" t="n"/>
       <c r="X27" s="26" t="n"/>
-      <c r="Y27" s="26" t="n"/>
+      <c r="Y27" s="55" t="n"/>
       <c r="Z27" s="10" t="n"/>
       <c r="AA27" s="10" t="n"/>
       <c r="AB27" s="25" t="n"/>
       <c r="AC27" s="10" t="n"/>
-      <c r="AD27" s="19" t="n"/>
+      <c r="AD27" s="55" t="n"/>
     </row>
     <row r="28" ht="24.9" customHeight="1">
       <c r="B28" s="46" t="n"/>
@@ -1819,12 +1864,12 @@
       <c r="V28" s="10" t="n"/>
       <c r="W28" s="10" t="n"/>
       <c r="X28" s="26" t="n"/>
-      <c r="Y28" s="26" t="n"/>
+      <c r="Y28" s="55" t="n"/>
       <c r="Z28" s="10" t="n"/>
       <c r="AA28" s="10" t="n"/>
       <c r="AB28" s="25" t="n"/>
       <c r="AC28" s="10" t="n"/>
-      <c r="AD28" s="19" t="n"/>
+      <c r="AD28" s="55" t="n"/>
     </row>
     <row r="29" ht="24.9" customHeight="1">
       <c r="B29" s="46" t="n"/>
@@ -1850,12 +1895,12 @@
       <c r="V29" s="10" t="n"/>
       <c r="W29" s="10" t="n"/>
       <c r="X29" s="26" t="n"/>
-      <c r="Y29" s="26" t="n"/>
+      <c r="Y29" s="55" t="n"/>
       <c r="Z29" s="10" t="n"/>
       <c r="AA29" s="10" t="n"/>
       <c r="AB29" s="25" t="n"/>
       <c r="AC29" s="10" t="n"/>
-      <c r="AD29" s="19" t="n"/>
+      <c r="AD29" s="55" t="n"/>
     </row>
     <row r="30" ht="21" customHeight="1">
       <c r="B30" s="46" t="n"/>
@@ -1881,12 +1926,12 @@
       <c r="V30" s="10" t="n"/>
       <c r="W30" s="10" t="n"/>
       <c r="X30" s="26" t="n"/>
-      <c r="Y30" s="26" t="n"/>
+      <c r="Y30" s="55" t="n"/>
       <c r="Z30" s="10" t="n"/>
       <c r="AA30" s="10" t="n"/>
       <c r="AB30" s="25" t="n"/>
       <c r="AC30" s="10" t="n"/>
-      <c r="AD30" s="19" t="n"/>
+      <c r="AD30" s="55" t="n"/>
     </row>
     <row r="31" ht="25.5" customHeight="1">
       <c r="B31" s="46" t="n"/>
@@ -1912,12 +1957,12 @@
       <c r="V31" s="10" t="n"/>
       <c r="W31" s="10" t="n"/>
       <c r="X31" s="26" t="n"/>
-      <c r="Y31" s="26" t="n"/>
+      <c r="Y31" s="55" t="n"/>
       <c r="Z31" s="10" t="n"/>
       <c r="AA31" s="10" t="n"/>
       <c r="AB31" s="25" t="n"/>
       <c r="AC31" s="10" t="n"/>
-      <c r="AD31" s="19" t="n"/>
+      <c r="AD31" s="55" t="n"/>
       <c r="AE31" s="2" t="n"/>
     </row>
     <row r="32" ht="25.5" customHeight="1">
@@ -1944,12 +1989,12 @@
       <c r="V32" s="10" t="n"/>
       <c r="W32" s="10" t="n"/>
       <c r="X32" s="26" t="n"/>
-      <c r="Y32" s="26" t="n"/>
+      <c r="Y32" s="55" t="n"/>
       <c r="Z32" s="10" t="n"/>
       <c r="AA32" s="10" t="n"/>
       <c r="AB32" s="25" t="n"/>
       <c r="AC32" s="10" t="n"/>
-      <c r="AD32" s="19" t="n"/>
+      <c r="AD32" s="55" t="n"/>
       <c r="AE32" s="2" t="n"/>
     </row>
     <row r="33" ht="25.5" customHeight="1">
@@ -1976,12 +2021,12 @@
       <c r="V33" s="10" t="n"/>
       <c r="W33" s="10" t="n"/>
       <c r="X33" s="26" t="n"/>
-      <c r="Y33" s="10" t="n"/>
+      <c r="Y33" s="55" t="n"/>
       <c r="Z33" s="10" t="n"/>
       <c r="AA33" s="10" t="n"/>
       <c r="AB33" s="25" t="n"/>
       <c r="AC33" s="10" t="n"/>
-      <c r="AD33" s="19" t="n"/>
+      <c r="AD33" s="55" t="n"/>
       <c r="AE33" s="2" t="n"/>
     </row>
     <row r="34" ht="25.5" customHeight="1">
@@ -2008,12 +2053,12 @@
       <c r="V34" s="10" t="n"/>
       <c r="W34" s="10" t="n"/>
       <c r="X34" s="26" t="n"/>
-      <c r="Y34" s="10" t="n"/>
+      <c r="Y34" s="55" t="n"/>
       <c r="Z34" s="10" t="n"/>
       <c r="AA34" s="10" t="n"/>
       <c r="AB34" s="25" t="n"/>
       <c r="AC34" s="10" t="n"/>
-      <c r="AD34" s="19" t="n"/>
+      <c r="AD34" s="55" t="n"/>
       <c r="AE34" s="2" t="n"/>
     </row>
     <row r="35" ht="25.5" customHeight="1">
@@ -2040,12 +2085,12 @@
       <c r="V35" s="10" t="n"/>
       <c r="W35" s="10" t="n"/>
       <c r="X35" s="26" t="n"/>
-      <c r="Y35" s="10" t="n"/>
+      <c r="Y35" s="55" t="n"/>
       <c r="Z35" s="10" t="n"/>
       <c r="AA35" s="10" t="n"/>
       <c r="AB35" s="25" t="n"/>
       <c r="AC35" s="10" t="n"/>
-      <c r="AD35" s="19" t="n"/>
+      <c r="AD35" s="55" t="n"/>
       <c r="AE35" s="2" t="n"/>
     </row>
     <row r="36" ht="25.5" customHeight="1">
@@ -2072,12 +2117,12 @@
       <c r="V36" s="10" t="n"/>
       <c r="W36" s="10" t="n"/>
       <c r="X36" s="26" t="n"/>
-      <c r="Y36" s="10" t="n"/>
+      <c r="Y36" s="55" t="n"/>
       <c r="Z36" s="10" t="n"/>
       <c r="AA36" s="10" t="n"/>
       <c r="AB36" s="25" t="n"/>
       <c r="AC36" s="10" t="n"/>
-      <c r="AD36" s="19" t="n"/>
+      <c r="AD36" s="55" t="n"/>
       <c r="AE36" s="2" t="n"/>
     </row>
     <row r="37" ht="25.5" customHeight="1">
@@ -2104,12 +2149,12 @@
       <c r="V37" s="10" t="n"/>
       <c r="W37" s="10" t="n"/>
       <c r="X37" s="26" t="n"/>
-      <c r="Y37" s="10" t="n"/>
+      <c r="Y37" s="55" t="n"/>
       <c r="Z37" s="10" t="n"/>
       <c r="AA37" s="10" t="n"/>
       <c r="AB37" s="10" t="n"/>
       <c r="AC37" s="10" t="n"/>
-      <c r="AD37" s="19" t="n"/>
+      <c r="AD37" s="55" t="n"/>
       <c r="AE37" s="2" t="n"/>
     </row>
     <row r="38" ht="25.5" customHeight="1">
@@ -2136,12 +2181,12 @@
       <c r="V38" s="10" t="n"/>
       <c r="W38" s="10" t="n"/>
       <c r="X38" s="26" t="n"/>
-      <c r="Y38" s="10" t="n"/>
+      <c r="Y38" s="55" t="n"/>
       <c r="Z38" s="10" t="n"/>
       <c r="AA38" s="10" t="n"/>
       <c r="AB38" s="10" t="n"/>
       <c r="AC38" s="10" t="n"/>
-      <c r="AD38" s="19" t="n"/>
+      <c r="AD38" s="55" t="n"/>
       <c r="AE38" s="2" t="n"/>
     </row>
     <row r="39" ht="25.5" customHeight="1">
@@ -2168,12 +2213,12 @@
       <c r="V39" s="10" t="n"/>
       <c r="W39" s="10" t="n"/>
       <c r="X39" s="26" t="n"/>
-      <c r="Y39" s="10" t="n"/>
+      <c r="Y39" s="55" t="n"/>
       <c r="Z39" s="10" t="n"/>
       <c r="AA39" s="10" t="n"/>
       <c r="AB39" s="10" t="n"/>
       <c r="AC39" s="10" t="n"/>
-      <c r="AD39" s="19" t="n"/>
+      <c r="AD39" s="55" t="n"/>
       <c r="AE39" s="2" t="n"/>
     </row>
     <row r="40" ht="25.5" customHeight="1">
@@ -2200,12 +2245,12 @@
       <c r="V40" s="32" t="n"/>
       <c r="W40" s="32" t="n"/>
       <c r="X40" s="26" t="n"/>
-      <c r="Y40" s="32" t="n"/>
+      <c r="Y40" s="55" t="n"/>
       <c r="Z40" s="32" t="n"/>
       <c r="AA40" s="32" t="n"/>
       <c r="AB40" s="32" t="n"/>
       <c r="AC40" s="32" t="n"/>
-      <c r="AD40" s="34" t="n"/>
+      <c r="AD40" s="55" t="n"/>
       <c r="AE40" s="2" t="n"/>
     </row>
     <row r="41" ht="25.5" customHeight="1">
@@ -2232,12 +2277,12 @@
       <c r="V41" s="32" t="n"/>
       <c r="W41" s="32" t="n"/>
       <c r="X41" s="26" t="n"/>
-      <c r="Y41" s="32" t="n"/>
+      <c r="Y41" s="55" t="n"/>
       <c r="Z41" s="32" t="n"/>
       <c r="AA41" s="32" t="n"/>
       <c r="AB41" s="32" t="n"/>
       <c r="AC41" s="32" t="n"/>
-      <c r="AD41" s="34" t="n"/>
+      <c r="AD41" s="55" t="n"/>
       <c r="AE41" s="2" t="n"/>
     </row>
     <row r="42" ht="25.5" customHeight="1">
@@ -2264,12 +2309,12 @@
       <c r="V42" s="32" t="n"/>
       <c r="W42" s="32" t="n"/>
       <c r="X42" s="26" t="n"/>
-      <c r="Y42" s="32" t="n"/>
+      <c r="Y42" s="55" t="n"/>
       <c r="Z42" s="32" t="n"/>
       <c r="AA42" s="32" t="n"/>
       <c r="AB42" s="32" t="n"/>
       <c r="AC42" s="32" t="n"/>
-      <c r="AD42" s="34" t="n"/>
+      <c r="AD42" s="55" t="n"/>
       <c r="AE42" s="2" t="n"/>
     </row>
     <row r="43" ht="25.5" customHeight="1">
@@ -2296,12 +2341,12 @@
       <c r="V43" s="32" t="n"/>
       <c r="W43" s="32" t="n"/>
       <c r="X43" s="26" t="n"/>
-      <c r="Y43" s="32" t="n"/>
+      <c r="Y43" s="55" t="n"/>
       <c r="Z43" s="32" t="n"/>
       <c r="AA43" s="32" t="n"/>
       <c r="AB43" s="32" t="n"/>
       <c r="AC43" s="32" t="n"/>
-      <c r="AD43" s="34" t="n"/>
+      <c r="AD43" s="55" t="n"/>
       <c r="AE43" s="2" t="n"/>
     </row>
     <row r="44" ht="25.5" customHeight="1">
@@ -2328,12 +2373,12 @@
       <c r="V44" s="32" t="n"/>
       <c r="W44" s="32" t="n"/>
       <c r="X44" s="26" t="n"/>
-      <c r="Y44" s="32" t="n"/>
+      <c r="Y44" s="55" t="n"/>
       <c r="Z44" s="32" t="n"/>
       <c r="AA44" s="32" t="n"/>
       <c r="AB44" s="32" t="n"/>
       <c r="AC44" s="32" t="n"/>
-      <c r="AD44" s="34" t="n"/>
+      <c r="AD44" s="55" t="n"/>
       <c r="AE44" s="2" t="n"/>
     </row>
     <row r="45" ht="25.5" customHeight="1">
@@ -2360,12 +2405,12 @@
       <c r="V45" s="32" t="n"/>
       <c r="W45" s="32" t="n"/>
       <c r="X45" s="26" t="n"/>
-      <c r="Y45" s="32" t="n"/>
+      <c r="Y45" s="55" t="n"/>
       <c r="Z45" s="32" t="n"/>
       <c r="AA45" s="32" t="n"/>
       <c r="AB45" s="32" t="n"/>
       <c r="AC45" s="32" t="n"/>
-      <c r="AD45" s="34" t="n"/>
+      <c r="AD45" s="55" t="n"/>
       <c r="AE45" s="2" t="n"/>
     </row>
     <row r="46" ht="25.5" customHeight="1">
@@ -2392,12 +2437,12 @@
       <c r="V46" s="32" t="n"/>
       <c r="W46" s="32" t="n"/>
       <c r="X46" s="26" t="n"/>
-      <c r="Y46" s="32" t="n"/>
+      <c r="Y46" s="55" t="n"/>
       <c r="Z46" s="32" t="n"/>
       <c r="AA46" s="32" t="n"/>
       <c r="AB46" s="32" t="n"/>
       <c r="AC46" s="32" t="n"/>
-      <c r="AD46" s="34" t="n"/>
+      <c r="AD46" s="55" t="n"/>
       <c r="AE46" s="2" t="n"/>
     </row>
     <row r="47" ht="25.5" customHeight="1" thickBot="1">
@@ -2424,12 +2469,12 @@
       <c r="V47" s="22" t="n"/>
       <c r="W47" s="22" t="n"/>
       <c r="X47" s="22" t="n"/>
-      <c r="Y47" s="22" t="n"/>
+      <c r="Y47" s="55" t="n"/>
       <c r="Z47" s="22" t="n"/>
       <c r="AA47" s="22" t="n"/>
       <c r="AB47" s="22" t="n"/>
       <c r="AC47" s="22" t="n"/>
-      <c r="AD47" s="24" t="n"/>
+      <c r="AD47" s="55" t="n"/>
       <c r="AE47" s="2" t="n"/>
     </row>
   </sheetData>

</xml_diff>